<commit_message>
Fix quoted work title rendering and data sync
</commit_message>
<xml_diff>
--- a/public/data/open-works.xlsx
+++ b/public/data/open-works.xlsx
@@ -247,7 +247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -262,6 +262,7 @@
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -325,6 +326,11 @@
           <t>image_alt</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>external_note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
@@ -387,6 +393,11 @@
           <t/>
         </is>
       </c>
+      <c r="M2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="2">
@@ -449,6 +460,11 @@
           <t/>
         </is>
       </c>
+      <c r="M3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr" s="2">
@@ -511,6 +527,11 @@
           <t/>
         </is>
       </c>
+      <c r="M4" t="inlineStr" s="2">
+        <is>
+          <t>현재는 브라우저 프리뷰만 제공됩니다. 인코딩과 파일 렌더 기능은 준비 중입니다.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="2">
@@ -573,6 +594,11 @@
           <t/>
         </is>
       </c>
+      <c r="M5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="2">
@@ -635,6 +661,11 @@
           <t/>
         </is>
       </c>
+      <c r="M6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="2">
@@ -697,6 +728,11 @@
           <t/>
         </is>
       </c>
+      <c r="M7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
@@ -759,6 +795,11 @@
           <t/>
         </is>
       </c>
+      <c r="M8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="2">
@@ -821,9 +862,14 @@
           <t/>
         </is>
       </c>
+      <c r="M9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:M9"/>
 </worksheet>
 </file>
 
@@ -871,7 +917,7 @@
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="57" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
@@ -950,7 +996,7 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t>Web App 이용하기</t>
+          <t>Web App(beta) 이용하기</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Move Splatify preview note into web app button
</commit_message>
<xml_diff>
--- a/public/data/open-works.xlsx
+++ b/public/data/open-works.xlsx
@@ -1,34 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="open-works" sheetId="1" r:id="rId1"/>
-    <sheet name="open-work-details" sheetId="2" r:id="rId2"/>
-    <sheet name="open-works-page" sheetId="3" r:id="rId3"/>
-    <sheet name="open-work-links" sheetId="4" r:id="rId4"/>
-    <sheet name="open-work-examples" sheetId="5" r:id="rId5"/>
-    <sheet name="open-work-manuals" sheetId="6" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-works" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-work-details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-works-page" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-work-links" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-work-examples" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open-work-manuals" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'open-works'!$A$1:$C$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'open-work-details'!$A$1:$M$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'open-works-page'!$A$1:$B$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'open-work-links'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'open-work-examples'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'open-work-manuals'!$A$1:$E$26</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <name val="Aptos"/>
       <sz val="11"/>
-      <name val="Aptos"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -62,179 +71,534 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="58" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>summary</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>맥북을 닫아도 잠자기 모드로 들어가지 않는 앱
 긴 바이브코딩 작업을 하거나 브금을 틀어놓을 때 좋습니다</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>/sleepless</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>SPLATIFY</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>사용자의 이미지/영상을 가우시안 스플래팅 느낌으로 인코딩해주는 웹앱</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>/splatify</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>다양한 비디오 파일을 간단하게 압축 인코딩하는 앱</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>/ffmochi</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>코딩작업하다 보면 금새 차오르는 컨텍스트 때문에 곤란할 때,
 새 채팅으로 깔끔하게 옮겨주는 제비 에이전트</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>/jebi-agent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>딸깍장표</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>영상의 모든 컷을 감지, 대표 컷을 추출해서 장표 문서로 만들어주는 에이전트</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>/ttalkkak-jangpyo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="2">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>딸깍클리닝</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>초상 이미지를 기준으로 클리닝 영역을 감지해서 마킹해서 문서화해주는 에이전트</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>/ttalkkak-cleaning</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">JEJU WAVE RADIO </t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>실시간 제주 바닷가의 파도 + 날씨를 앰비언스 사운드 맵핑한 작업
 귀여운 8bit 영상도 함께 플레이</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>/jeju-wave-radio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="2">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>INTERACTIVE VISUALS</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="2">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>재미있는 인터랙티브 비주얼 프로젝트들</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="2">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>/interactive-visuals</t>
         </is>
@@ -242,665 +606,579 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="53" customWidth="1"/>
-    <col min="8" max="8" width="58" customWidth="1"/>
-    <col min="9" max="9" width="54" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="46" customWidth="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="53" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>kicker</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>detail_summary</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>format</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>lede</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>features</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>action_label</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>image_alt</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>external_note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Mac utility</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>맥북을 닫아도 잠자기 모드로 들어가지 않는 앱. 긴 바이브코딩 작업이나 음악 재생을 끊기지 않게 유지합니다.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Menu bar app</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Prototype</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS는 맥북 화면을 닫아도 작업 흐름이 멈추지 않도록 돕는 작은 유틸리티입니다.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr" s="2">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>긴 생성 작업, 로컬 서버, 음악 재생처럼 중간에 끊기면 불편한 상황을 위해 만들었습니다. 복잡한 설정 대신 켜고 끄는 상태가 즉시 보이고, 작업 중인 맥의 리듬을 방해하지 않는 조용한 인터페이스를 목표로 합니다.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="2">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>닫아도 유지되는 작업 세션|상태가 분명한 메뉴바 컨트롤|바이브코딩과 장시간 렌더링에 맞춘 흐름</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr" s="2">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>jeju-wave-radio</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Ambient web radio</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>실시간 제주 바닷가의 파도와 날씨를 앰비언스 사운드로 맵핑하고, 귀여운 8bit 영상과 함께 플레이합니다.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Web player</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Creative coding</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>JEJU WAVE RADIO 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr" s="2">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>실시간 파도, 날씨 데이터, 앰비언스 사운드 맵핑 구조를 차분히 묶고 있습니다. 조금만 기다려주세요. 응원의 메시지를 남겨주시면 다음 정리에 힘이 됩니다.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr" s="2">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr" s="2">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>splatify</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Gaussian-style encoder</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>이미지와 영상을 가우시안 스타일 포인트 비주얼로 변환하는 웹앱입니다.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Web app</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Local MVP</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr" s="2">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="2">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>SPLATIFY는 이미지와 영상을 가우시안 스타일의 포인트 비주얼로 변환하는 웹앱입니다.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr" s="2">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>JPG, PNG, MP4를 올려 브라우저에서 바로 프리뷰하고, 필요한 경우 MP4나 PNG로 출력하는 실험용 도구입니다.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr" s="2">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>이미지/영상 업로드 기반 변환|브라우저 WebGL 프리뷰|MP4/PNG 출력 흐름</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr" s="2">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr" s="2">
-        <is>
-          <t>현재는 브라우저 프리뷰만 제공됩니다. 인코딩과 파일 렌더 기능은 준비 중입니다.</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Video compression app</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>영상 파일 용량을 간단하게 줄여주는 macOS 앱입니다.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Desktop app</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Private test</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="2">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI는 macOS에서 영상 파일 용량을 가볍게 줄여주는 작은 앱입니다.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr" s="2">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>파일을 넣고 프리셋을 고르면 원본 옆에 압축된 MP4를 새로 만들어줍니다. 원본은 보존하고, 반복 인코딩을 부담 없이 끝내는 흐름을 목표로 합니다.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr" s="2">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>MP4/MOV/M4V 드래그 앤 드롭|상황에 맞춘 압축 프리셋|원본 보존과 새 MP4 출력</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr" s="2">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Codex handoff agent</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>긴 Codex 작업을 새 채팅으로 넘기는 제비 handoff Agent Skill입니다.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Agent Skill</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Personal utility</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="2">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Workflow design</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="2">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>무거워진 채팅을 접고, 작업은 이어갑니다.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr" s="2">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>JEBI는 현재 저장소 상태를 짧은 handoff로 압축하고 clean successor chat을 시작합니다. 전체 history를 복사하지 않고 repo, branch, HEAD, worktree, 변경 파일, 완료/남은 일, 테스트 상태, 주의사항만 넘깁니다. 다음 에이전트는 handoff와 live repo를 비교한 뒤 불일치를 보고하고 사용자 지시를 기다립니다.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="2">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>handoff 생성|clean successor chat|repo 상태 검증</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="2">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="2">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>interactive-visuals</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Interactive archive</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>재미있는 인터랙티브 비주얼 프로젝트들을 모아두는 실험실형 페이지입니다.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Project archive</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="2">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr" s="2">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Interaction design</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="2">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>INTERACTIVE VISUALS 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr" s="2">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>데모, 제작 맥락, 조작 방식까지 한 번에 볼 수 있도록 조금만 기다려주세요. 정리가 끝나면 인터랙션 기반 비주얼 실험을 짧은 모듈 단위로 살펴볼 수 있게 열어둘 예정입니다.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr" s="2">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="2">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ttalkkak-jangpyo</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Deck automation</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>영상의 모든 컷을 감지하고 대표 컷을 추출해서 장표 문서로 만들어주는 에이전트.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>AI agent</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="2">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr" s="2">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Workflow design</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr" s="2">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>딸깍장표 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr" s="2">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>실제 사용 흐름, 출력 예시, 검증 기준을 차근차근 묶고 있습니다. 조금만 기다려주세요. 먼저 궁금한 점이나 응원의 메시지를 남겨주시면 이후 페이지 구성에 반영하겠습니다.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr" s="2">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="2">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="2">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ttalkkak-cleaning</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="2">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Image review agent</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="2">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>초상 이미지를 기준으로 클리닝 영역을 감지해서 마킹하고 문서화해주는 에이전트.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="2">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>AI agent</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="2">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr" s="2">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Review system</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr" s="2">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>딸깍클리닝 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr" s="2">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>클리닝 체크 기준, 마킹 예시, 문서화 흐름을 보기 좋게 정리하는 중입니다. 조금만 기다려주세요. 응원의 메시지나 궁금한 점을 보내주시면 다음 업데이트에 참고하겠습니다.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr" s="2">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr" s="2">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Open Works</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>다양한 작업들의 아카이빙 및 실험실 공간입니다.</t>
         </is>
@@ -908,169 +1186,174 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="57" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sort</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Github 페이지 연결</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>https://github.com/kyutomatte/sleepless/</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MAC OS용 다운로드</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>/assets/downloads/sleepless/Sleepless_0.1.2_aarch64.dmg</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>splatify</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Web App(beta) 이용하기</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>/splatify-webapp</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>GitHub 페이지 연결</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>https://github.com/kyutomatte/ffMOCHI</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>MAC OS용 다운로드</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>/assets/downloads/ffmochi/ffMOCHI-local.dmg</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="2">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Github 페이지 연결</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>https://github.com/kyutomatte/jebi_agent</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1078,129 +1361,130 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="56" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>kicker</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>media_url</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>media_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>caption</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>sort</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>splatify</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Splatify demo</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>/assets/open-works/splatify/splatify-demo.mov</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>video</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Usage example</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>제비 요청 인식</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>/assets/open-works/jebi-agent/jebi-usage-example.png</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>image</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>사용자가 제비로 이사갈게요라고 말하면 JEBI 요청으로 인식하고 handoff 절차를 시작합니다.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1208,444 +1492,449 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>section_title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>step_title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>body</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>sort</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>설치하기</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>GitHub Releases 또는 MAC OS용 다운로드 버튼에서 Apple Silicon Mac용 DMG를 받은 뒤 Sleepless.app을 Applications 폴더로 옮겨주세요.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>처음 실행 허용하기</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>개인이 테스트 배포하는 빌드라 아직 Apple 공식 개발자 서명과 공증이 적용되어 있지 않습니다. 안전한 배포 절차를 준비 중이니 처음 실행 시 macOS 보안 안내가 나타날 수 있습니다. 먼저 Done을 눌러 경고창을 닫고, System Settings &gt; Privacy &amp; Security에서 Open Anyway를 선택해주세요. 완료를 누른 뒤 시스템 설정 &gt; 개인정보 보호 및 보안에서 그래도 열기를 선택하면 실행할 수 있습니다. macOS 버전에 따라 버튼 이름이 조금 다를 수 있습니다.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>전원 연결 확인하기</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS는 AC 전원 연결 상태에서만 awake mode를 켤 수 있습니다. 전원이 빠지면 배터리 보호를 위해 모드가 자동으로 종료됩니다.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>잠자기 방지 켜기</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>메뉴바의 8bit 유령 아이콘에서 잠자기 방지를 켭니다. 처음 켤 때는 closed-lid sleep 제어를 위한 관리자 인증이 한 번 필요할 수 있습니다.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>유지 시간 고르기</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>닫힌 상태 유지 시간을 10분, 30분, 1시간, 영구 중에서 고를 수 있습니다. 뚜껑을 닫으면 밝기를 0으로 낮추고, 다시 열거나 모드를 끄면 이전 밝기를 복구합니다.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="2">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>sleepless</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SLEEPLESS Manual</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>문제 시 복구하기</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>앱이 비정상 종료된 뒤 닫힘 잠자기가 돌아오지 않으면 터미널에서 sudo pmset -c disablesleep 0 명령으로 macOS 기본 전원 설정을 복구할 수 있습니다.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="2">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>설치하기</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>MAC OS용 다운로드 버튼에서 ffMOCHI-local.dmg를 받은 뒤 ffMOCHI.app을 Applications 폴더로 드래그해주세요.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="2">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="2">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="2">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="2">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>처음 실행 허용하기</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="2">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>개인이 테스트 배포하는 빌드라 아직 Apple 공식 개발자 서명과 공증이 적용되어 있지 않습니다. 안전한 배포 절차를 준비 중이니 처음 실행 시 macOS 보안 안내가 나타날 수 있습니다. 먼저 Done을 눌러 경고창을 닫고, System Settings &gt; Privacy &amp; Security에서 Open Anyway를 선택해주세요. 완료를 누른 뒤 시스템 설정 &gt; 개인정보 보호 및 보안에서 그래도 열기를 선택하면 실행할 수 있습니다. macOS 버전에 따라 버튼 이름이 조금 다를 수 있습니다.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="2">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="2">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="2">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>FFmpeg 준비하기</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="2">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI는 로컬 FFmpeg로 영상을 압축합니다. 앱에 설치 안내가 보이면 Homebrew에서 brew install ffmpeg를 실행한 뒤 CHECK AGAIN을 눌러주세요.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="2">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr" s="2">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr" s="2">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="2">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>영상 넣고 시작하기</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr" s="2">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>MP4 MOV M4V 파일을 앱 창에 드래그하거나 앱 아이콘 위에 드롭한 뒤 프리셋을 고르고 START를 누르면 압축이 시작됩니다.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="2">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr" s="2">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr" s="2">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="2">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>출력 확인하기</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="2">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>완료된 파일은 원본 옆에 OriginalName_compressed.mp4 형태로 저장됩니다. 같은 이름이 있으면 _compressed_001.mp4처럼 번호를 붙여 덮어쓰지 않습니다.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="2">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr" s="2">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>ffmochi</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="2">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>ffMOCHI Manual</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="2">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>문제 시 확인하기</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="2">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>압축이 실패하면 FFmpeg 설치, 지원 파일 형식, 출력 폴더 권한, 디스크 공간을 확인해주세요. Default MP4로 다시 시도하기 전 일부만 만들어진 _compressed.mp4 파일이 남아 있으면 삭제하는 것이 좋습니다.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="2">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr" s="2">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="2">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="2">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>왜 필요한가</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="2">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>긴 코딩 채팅이 무거워지고 컨텍스트가 길어져 결정이 묻히기 시작할 때 씁니다. Fork는 너무 많은 history를 복사하고, 완전히 새로 시작하면 맥락을 잃습니다. JEBI는 그 중간 지점에서 현재 작업 상태만 압축해 새 채팅으로 넘깁니다.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="2">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr" s="2">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="2">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>설치와 발동</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="2">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>가장 쉬운 설치 방법은 GitHub 주소와 README를 에이전트에게 전달하는 것입니다. 단, 주소만 주는 방식은 해당 대화 안에서 읽고 따라 하는 것에 가깝습니다. 다음 대화에서도 자동으로 JEBI가 발동되게 하려면 사용하는 도구가 지원하는 Skills, 프로젝트 지침, custom instruction 중 하나에 등록해야 합니다.
 PROMPT: https://github.com/kyutomatte/jebi_agent 확인하고 README.md 기준으로 설치와 사용 방법을 알려주세요.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr" s="2">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr" s="2">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr" s="2">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr" s="2">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>환경별 설치 방법</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr" s="2">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>환경|가장 쉬운 방법|계속 쓰는 방법|발동 문구
 ChatGPT / GPT|GitHub 주소와 README.md를 읽어 달라고 합니다.|지원되는 Skills/프로젝트 지침 환경이면 Skill 폴더 또는 SKILL.md 핵심 규칙을 등록하고, 일반 ChatGPT/GPT에서는 Custom Instructions, GPT 지침, 프로젝트 지침에 핵심 규칙을 붙입니다.|$jebi 또는 제비로 옮겨주세요
@@ -1656,29 +1945,29 @@
 기타 LLM|GitHub 주소를 주고 README.md를 따라 하게 합니다.|system/custom instruction, 프로젝트 지침, 지식 베이스에 SKILL.md 핵심을 넣습니다.|JEBI 모드로 정리해줘</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr" s="2">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr" s="2">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr" s="2">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="2">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>터미널 설치</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="2">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>터미널에서 쓰는 에이전트는 설치 스크립트가 가장 단순합니다.
 CMD: scripts/install-skill.sh codex
@@ -1693,29 +1982,29 @@
 지침, custom command, 프로젝트 rule은 설치할 수 있지만 Codex Desktop thread API가 생기지는 않습니다.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr" s="2">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr" s="2">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr" s="2">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr" s="2">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>호출 예시</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr" s="2">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>유형|예시|설명
 실행어 호출 예시|$jebi|현재 작업을 새 Codex 채팅으로 넘기는 JEBI handoff를 시작합니다.
@@ -1727,58 +2016,58 @@
 오작동 방지|파일명 jebi 또는 동물 제비 이야기|새 채팅 이동 의도가 없으면 실행하지 않습니다.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr" s="2">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr" s="2">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="2">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="2">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>자동으로 넘기는 정보</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="2">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>JEBI는 현재 repository, branch, HEAD, worktree 상태를 먼저 확인합니다.
 handoff에는 전체 diff가 아니라 변경 파일 요약, 완료한 일과 남은 일, 중요한 결정, 바꾸면 안 되는 내용이 들어갑니다.
 test/build/lint/typecheck 상태, 적용되는 AGENTS.md 지침, known failure recovery note도 함께 정리합니다.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr" s="2">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr" s="2">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr" s="2">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="2">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>작동 방식</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr" s="2">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>실행되면 .codex/handoffs/NNN-handoff.md를 만들고 latest.md를 갱신합니다.
 state.json은 retry와 numbering을 위한 로컬 상태로 남깁니다.
@@ -1786,181 +2075,181 @@
 새 채팅에는 handoff 경로와 확인 지시만 보냅니다.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr" s="2">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr" s="2">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="2">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr" s="2">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>새 채팅 이름</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr" s="2">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>새 채팅 이름은 프로젝트 폴더명이 아니라 현재 작업 제목을 기준으로 붙입니다. 예를 들어 UI UX에서 처음 옮기면 UI UX #02가 됩니다.
 거기서 다시 옮기면 UI UX #02 #02가 아니라 UI UX #03이 됩니다.
 제목을 읽을 수 없으면 project name으로 대체하지 않습니다.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr" s="2">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr" s="2">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr" s="2">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr" s="2">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>새 채팅에서 먼저 하는 일</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr" s="2">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>successor 에이전트는 handoff 파일을 읽고 실제 repo와 비교합니다.
 브랜치, 워킹트리, 변경 파일, 누락된 맥락이 맞는지 확인하고, 불일치가 있으면 먼저 보고합니다.
 그 전에는 파일을 수정하지 않고 사용자 지시를 기다립니다.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr" s="2">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr" s="2">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr" s="2">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr" s="2">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Dirty 상태 다루기</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr" s="2">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>JEBI는 .codex/handoffs 안에 markdown handoff를 만들기 때문에 실행 직후 dirty 상태가 생길 수 있습니다.
 handoff만 바뀌었다면 Clean except JEBI handoff artifacts로 보고합니다.
 실제 프로젝트 변경과 섞여 있다면 Dirty: project changes + JEBI handoff artifacts로 구분합니다.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr" s="2">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr" s="2">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr" s="2">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr" s="2">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>주의점</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr" s="2">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>JEBI는 fork가 아닙니다. 현재 채팅을 복제하는 대신 clean successor chat을 시작합니다.
 전체 이전 채팅 history를 복사하지 않고, AppleScript, 화면 좌표 클릭, 내부 DB 수정, undocumented UI API 같은 우회도 쓰지 않아야 합니다.
 실제 저장소 상태가 대화 기억보다 우선입니다.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr" s="2">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr" s="2">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr" s="2">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr" s="2">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>보안 규칙</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr" s="2">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>handoff에는 API keys, tokens, cookies, authorization headers, .env values 같은 민감한 정보를 넣지 않습니다.
 의심되는 값은 REDACTED로 치환합니다.
 파괴적인 git 명령은 사용자 승인 없이 실행하지 않고, 새 채팅이 보이지 않으면 성공으로 말하지 않습니다.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr" s="2">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr" s="2">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>jebi-agent</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr" s="2">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>JEBI AGENT Tutorial</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr" s="2">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>테스트와 삭제</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr" s="2">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>개발자는 python3 -m unittest discover -s tests -v로 루트 테스트를 돌립니다.
 Skill 번들 테스트는 python3 -m unittest discover -s skill/jebi-agent/tests -v로 확인합니다.
 삭제할 때는 rm -rf ~/.codex/skills/jebi-agent 와 rm -rf ~/.codex/skills/jebi를 실행합니다. 프로젝트의 handoff 파일은 별도로 남습니다.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr" s="2">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -1968,5 +2257,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add bilingual portfolio support
</commit_message>
<xml_diff>
--- a/public/data/open-works.xlsx
+++ b/public/data/open-works.xlsx
@@ -76,12 +76,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="58" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -92,10 +94,20 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
+          <t>title_en</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
           <t>summary</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>summary_en</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>slug</t>
         </is>
@@ -109,11 +121,21 @@
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
           <t>맥북을 닫아도 잠자기 모드로 들어가지 않는 앱
 긴 바이브코딩 작업을 하거나 브금을 틀어놓을 때 좋습니다</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t>Keeps your Mac awake with the lid closed.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="2">
         <is>
           <t>/sleepless</t>
         </is>
@@ -127,10 +149,20 @@
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
+          <t>SPLATIFY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
           <t>사용자의 이미지/영상을 가우시안 스플래팅 느낌으로 인코딩해주는 웹앱</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>Turns images and videos into Gaussian-splatting-style visuals.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
         <is>
           <t>/splatify</t>
         </is>
@@ -144,10 +176,20 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
           <t>다양한 비디오 파일을 간단하게 압축 인코딩하는 앱</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>Compresses common video files with a simple workflow.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
         <is>
           <t>/ffmochi</t>
         </is>
@@ -161,11 +203,21 @@
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
           <t>코딩작업하다 보면 금새 차오르는 컨텍스트 때문에 곤란할 때,
 새 채팅으로 깔끔하게 옮겨주는 제비 에이전트</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t>Moves your work into a clean new chat before coding context fills up.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
         <is>
           <t>/jebi-agent</t>
         </is>
@@ -179,10 +231,20 @@
       </c>
       <c r="B6" t="inlineStr" s="2">
         <is>
+          <t>TTALKKAK DECK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
           <t>영상의 모든 컷을 감지, 대표 컷을 추출해서 장표 문서로 만들어주는 에이전트</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t>Detects video cuts and turns representative frames into a presentation deck.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
         <is>
           <t>/ttalkkak-jangpyo</t>
         </is>
@@ -196,10 +258,20 @@
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
+          <t>TTALKKAK CLEANING</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
           <t>초상 이미지를 기준으로 클리닝 영역을 감지해서 마킹해서 문서화해주는 에이전트</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t>Finds and marks portrait cleanup areas for a documented review.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
         <is>
           <t>/ttalkkak-cleaning</t>
         </is>
@@ -213,11 +285,21 @@
       </c>
       <c r="B8" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">JEJU WAVE RADIO </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
           <t>실시간 제주 바닷가의 파도 + 날씨를 앰비언스 사운드 맵핑한 작업
 귀여운 8bit 영상도 함께 플레이</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t>Maps live Jeju waves and weather to ambient sound and 8-bit visuals.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
         <is>
           <t>/jeju-wave-radio</t>
         </is>
@@ -231,38 +313,59 @@
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
+          <t>INTERACTIVE VISUALS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
           <t>재미있는 인터랙티브 비주얼 프로젝트들</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="2">
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t>A collection of playful interactive visual experiments.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
         <is>
           <t>/interactive-visuals</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C9"/>
+  <autoFilter ref="A1:E9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="58" customWidth="1"/>
-    <col min="8" max="8" width="58" customWidth="1"/>
-    <col min="9" max="9" width="54" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+    <col min="5" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="58" customWidth="1"/>
+    <col min="13" max="13" width="58" customWidth="1"/>
+    <col min="14" max="14" width="58" customWidth="1"/>
+    <col min="15" max="15" width="58" customWidth="1"/>
+    <col min="16" max="16" width="54" customWidth="1"/>
+    <col min="17" max="17" width="58" customWidth="1"/>
+    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="19" max="19" width="29" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
+    <col min="21" max="21" width="12" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="15" customWidth="1"/>
+    <col min="24" max="24" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -278,57 +381,112 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>kicker_en</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>detail_summary</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>detail_summary_en</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>format</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>format_en</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>status_en</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>role_en</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t>lede</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>lede_en</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t>detail</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t>detail_en</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
         <is>
           <t>features</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t>features_en</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
         <is>
           <t>action_label</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t>action_label_en</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr" s="1">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="1">
         <is>
           <t>image_alt</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="1">
+        <is>
+          <t>image_alt_en</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr" s="1">
         <is>
           <t>external_note</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr" s="1">
+        <is>
+          <t>external_note_en</t>
         </is>
       </c>
     </row>
@@ -345,55 +503,110 @@
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
+          <t>Mac utility</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
           <t>맥북을 닫아도 잠자기 모드로 들어가지 않는 앱. 긴 바이브코딩 작업이나 음악 재생을 끊기지 않게 유지합니다.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="E2" t="inlineStr" s="2">
+        <is>
+          <t>An app that keeps your Mac awake with the lid closed, so long vibe-coding jobs and music playback continue uninterrupted.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
         <is>
           <t>Menu bar app</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t>Menu bar app</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="2">
         <is>
           <t>Prototype</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="I2" t="inlineStr" s="2">
+        <is>
+          <t>Prototype</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="2">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="K2" t="inlineStr" s="2">
+        <is>
+          <t>Design / Build</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr" s="2">
         <is>
           <t>SLEEPLESS는 맥북 화면을 닫아도 작업 흐름이 멈추지 않도록 돕는 작은 유틸리티입니다.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr" s="2">
+      <c r="M2" t="inlineStr" s="2">
+        <is>
+          <t>SLEEPLESS is a small utility that keeps your workflow moving even when you close your MacBook.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr" s="2">
         <is>
           <t>긴 생성 작업, 로컬 서버, 음악 재생처럼 중간에 끊기면 불편한 상황을 위해 만들었습니다. 복잡한 설정 대신 켜고 끄는 상태가 즉시 보이고, 작업 중인 맥의 리듬을 방해하지 않는 조용한 인터페이스를 목표로 합니다.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="2">
+      <c r="O2" t="inlineStr" s="2">
+        <is>
+          <t>It was made for long generation jobs, local servers, music playback, and other situations where an interruption is inconvenient. Instead of complex settings, it aims for a quiet interface that makes its on/off state immediately clear and stays out of your Mac workflow.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr" s="2">
         <is>
           <t>닫아도 유지되는 작업 세션|상태가 분명한 메뉴바 컨트롤|바이브코딩과 장시간 렌더링에 맞춘 흐름</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr" s="2">
+      <c r="Q2" t="inlineStr" s="2">
+        <is>
+          <t>Work sessions that continue with the lid closed|Clear menu bar controls|A flow designed for vibe coding and long renders</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr" s="2">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr" s="2">
+      <c r="S2" t="inlineStr" s="2">
+        <is>
+          <t>Send feedback or an inquiry</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -412,55 +625,110 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
+          <t>Ambient web radio</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
           <t>실시간 제주 바닷가의 파도와 날씨를 앰비언스 사운드로 맵핑하고, 귀여운 8bit 영상과 함께 플레이합니다.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>Maps live waves and weather from the Jeju coast to ambient sound and plays it with a cute 8-bit animation.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
         <is>
           <t>Web player</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t>Web player</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="2">
         <is>
           <t>ON AIR</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
+      <c r="I3" t="inlineStr" s="2">
+        <is>
+          <t>ON AIR</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="2">
         <is>
           <t>Creative coding</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="K3" t="inlineStr" s="2">
+        <is>
+          <t>Creative coding</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr" s="2">
         <is>
           <t>JEJU WAVE RADIO는 제주 바닷가의 파도와 날씨를 실시간 분위기로 엮어내는 웹 라디오입니다.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr" s="2">
+      <c r="M3" t="inlineStr" s="2">
+        <is>
+          <t>JEJU WAVE RADIO is a web radio project that weaves live waves and weather from the Jeju coast into a real-time atmosphere.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr" s="2">
         <is>
           <t>파도, 날씨, 시간대의 감각을 앰비언스 사운드와 귀여운 8bit 비주얼로 연결하는 작업입니다. 실제 플레이어 페이지는 별도로 열어두고, 상세 페이지에서는 프로젝트 소개와 시연 영상을 먼저 확인할 수 있습니다.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr" s="2">
+      <c r="O3" t="inlineStr" s="2">
+        <is>
+          <t>The project connects the feel of waves, weather, and time of day with ambient sound and cute 8-bit visuals. The live player opens separately, while this detail page introduces the project and its demo video.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr" s="2">
         <is>
           <t>실시간 자연 데이터|앰비언스 사운드 맵핑|8bit 비주얼 플레이어</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr" s="2">
+      <c r="Q3" t="inlineStr" s="2">
+        <is>
+          <t>Live nature data|Ambient sound mapping|8-bit visual player</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr" s="2">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr" s="2">
+      <c r="S3" t="inlineStr" s="2">
+        <is>
+          <t>Send feedback or an inquiry</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -479,55 +747,110 @@
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
+          <t>Gaussian-style encoder</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
           <t>이미지와 영상을 가우시안 스타일 포인트 비주얼로 변환하는 웹앱입니다.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>A web app that transforms images and videos into Gaussian-style point visuals.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
         <is>
           <t>Web app</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t>Web app</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
         <is>
           <t>Local MVP</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr" s="2">
+      <c r="I4" t="inlineStr" s="2">
+        <is>
+          <t>Local MVP</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="2">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="2">
+      <c r="K4" t="inlineStr" s="2">
+        <is>
+          <t>Design / Build</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr" s="2">
         <is>
           <t>SPLATIFY는 이미지와 영상을 가우시안 스타일의 포인트 비주얼로 변환하는 웹앱입니다.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr" s="2">
+      <c r="M4" t="inlineStr" s="2">
+        <is>
+          <t>SPLATIFY is a web app that transforms images and videos into Gaussian-style point visuals.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr" s="2">
         <is>
           <t>JPG, PNG, MP4를 올려 브라우저에서 바로 프리뷰하고, 필요한 경우 MP4나 PNG로 출력하는 실험용 도구입니다.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr" s="2">
+      <c r="O4" t="inlineStr" s="2">
+        <is>
+          <t>Upload a JPG, PNG, or MP4 to preview it directly in the browser, then export an MP4 or PNG when needed. It is an experimental tool for exploring this workflow.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr" s="2">
         <is>
           <t>이미지/영상 업로드 기반 변환|브라우저 WebGL 프리뷰|MP4/PNG 출력 흐름</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr" s="2">
+      <c r="Q4" t="inlineStr" s="2">
+        <is>
+          <t>Image and video upload conversion|WebGL preview in the browser|MP4/PNG export flow</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr" s="2">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr" s="2">
+      <c r="S4" t="inlineStr" s="2">
+        <is>
+          <t>Send feedback or an inquiry</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -546,55 +869,110 @@
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
+          <t>Video compression app</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
           <t>영상 파일 용량을 간단하게 줄여주는 macOS 앱입니다.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t>A macOS app that makes it easy to reduce video file sizes.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
         <is>
           <t>Desktop app</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="G5" t="inlineStr" s="2">
+        <is>
+          <t>Desktop app</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="2">
         <is>
           <t>Private test</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="I5" t="inlineStr" s="2">
+        <is>
+          <t>Private test</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="2">
         <is>
           <t>Design / Build</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="2">
+      <c r="K5" t="inlineStr" s="2">
+        <is>
+          <t>Design / Build</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr" s="2">
         <is>
           <t>ffMOCHI는 macOS에서 영상 파일 용량을 가볍게 줄여주는 작은 앱입니다.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr" s="2">
+      <c r="M5" t="inlineStr" s="2">
+        <is>
+          <t>ffMOCHI is a small macOS app for lightly reducing video file sizes.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr" s="2">
         <is>
           <t>파일을 넣고 프리셋을 고르면 원본 옆에 압축된 MP4를 새로 만들어줍니다. 원본은 보존하고, 반복 인코딩을 부담 없이 끝내는 흐름을 목표로 합니다.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr" s="2">
+      <c r="O5" t="inlineStr" s="2">
+        <is>
+          <t>Drop in a file and choose a preset to create a compressed MP4 beside the original. The original stays untouched, and the workflow is designed to make repeated encoding painless.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr" s="2">
         <is>
           <t>MP4/MOV/M4V 드래그 앤 드롭|상황에 맞춘 압축 프리셋|원본 보존과 새 MP4 출력</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr" s="2">
+      <c r="Q5" t="inlineStr" s="2">
+        <is>
+          <t>MP4/MOV/M4V drag and drop|Compression presets for different needs|Original preservation with a new MP4 output</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr" s="2">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr" s="2">
+      <c r="S5" t="inlineStr" s="2">
+        <is>
+          <t>Send feedback or an inquiry</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -613,55 +991,110 @@
       </c>
       <c r="C6" t="inlineStr" s="2">
         <is>
+          <t>Codex handoff agent</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
           <t>긴 Codex 작업을 새 채팅으로 넘기는 제비 handoff Agent Skill입니다.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t>A JEBI handoff Agent Skill that moves a long Codex task into a new chat.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
         <is>
           <t>Agent Skill</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="G6" t="inlineStr" s="2">
+        <is>
+          <t>Agent Skill</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="2">
         <is>
           <t>Personal utility</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="2">
+      <c r="I6" t="inlineStr" s="2">
+        <is>
+          <t>Personal utility</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="2">
         <is>
           <t>Workflow design</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="2">
+      <c r="K6" t="inlineStr" s="2">
+        <is>
+          <t>Workflow design</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr" s="2">
         <is>
           <t>무거워진 채팅을 접고, 작업은 이어갑니다.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr" s="2">
+      <c r="M6" t="inlineStr" s="2">
+        <is>
+          <t>Close the overloaded chat and keep the work moving.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr" s="2">
         <is>
           <t>JEBI는 현재 저장소 상태를 짧은 handoff로 압축하고 clean successor chat을 시작합니다. 전체 history를 복사하지 않고 repo, branch, HEAD, worktree, 변경 파일, 완료/남은 일, 테스트 상태, 주의사항만 넘깁니다. 다음 에이전트는 handoff와 live repo를 비교한 뒤 불일치를 보고하고 사용자 지시를 기다립니다.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="2">
+      <c r="O6" t="inlineStr" s="2">
+        <is>
+          <t>JEBI compresses the current repository state into a short handoff and starts a clean successor chat. Rather than copying the entire history, it carries over only the repo, branch, HEAD, worktree, changed files, completed and remaining work, test status, and cautions. The next agent compares the handoff with the live repo, reports any mismatch, and waits for user direction.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr" s="2">
         <is>
           <t>handoff 생성|clean successor chat|repo 상태 검증</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="2">
+      <c r="Q6" t="inlineStr" s="2">
+        <is>
+          <t>Handoff generation|Clean successor chat|Repository state verification</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr" s="2">
         <is>
           <t>피드백 및 문의 작성</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr" s="2">
+      <c r="S6" t="inlineStr" s="2">
+        <is>
+          <t>Send feedback or an inquiry</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -680,55 +1113,110 @@
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
+          <t>Interactive archive</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
           <t>재미있는 인터랙티브 비주얼 프로젝트들을 모아두는 실험실형 페이지입니다.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t>A lab-style page that collects playful interactive visual projects.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
         <is>
           <t>Project archive</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="2">
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t>Project archive</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="2">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr" s="2">
+      <c r="I7" t="inlineStr" s="2">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="2">
         <is>
           <t>Interaction design</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="2">
+      <c r="K7" t="inlineStr" s="2">
+        <is>
+          <t>Interaction design</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr" s="2">
         <is>
           <t>INTERACTIVE VISUALS 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr" s="2">
+      <c r="M7" t="inlineStr" s="2">
+        <is>
+          <t>The INTERACTIVE VISUALS detail page is currently being organized.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr" s="2">
         <is>
           <t>데모, 제작 맥락, 조작 방식까지 한 번에 볼 수 있도록 조금만 기다려주세요. 정리가 끝나면 인터랙션 기반 비주얼 실험을 짧은 모듈 단위로 살펴볼 수 있게 열어둘 예정입니다.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr" s="2">
+      <c r="O7" t="inlineStr" s="2">
+        <is>
+          <t>Please wait a little longer while the demos, production context, and controls are brought together in one place. Once ready, the page will present interaction-driven visual experiments as short modules.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr" s="2">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="2">
+      <c r="Q7" t="inlineStr" s="2">
+        <is>
+          <t>Under construction|Please wait a little longer|A message of support makes a big difference to the next update</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr" s="2">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr" s="2">
+      <c r="S7" t="inlineStr" s="2">
+        <is>
+          <t>Send a message of support</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -747,55 +1235,110 @@
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
+          <t>Deck automation</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
           <t>영상의 모든 컷을 감지하고 대표 컷을 추출해서 장표 문서로 만들어주는 에이전트.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t>An agent that detects every cut in a video, extracts representative frames, and turns them into a presentation deck.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
         <is>
           <t>AI agent</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="2">
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t>AI agent</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="2">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr" s="2">
+      <c r="I8" t="inlineStr" s="2">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="2">
         <is>
           <t>Workflow design</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr" s="2">
+      <c r="K8" t="inlineStr" s="2">
+        <is>
+          <t>Workflow design</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr" s="2">
         <is>
           <t>딸깍장표 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr" s="2">
+      <c r="M8" t="inlineStr" s="2">
+        <is>
+          <t>The TTALKKAK DECK detail page is currently being organized.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr" s="2">
         <is>
           <t>실제 사용 흐름, 출력 예시, 검증 기준을 차근차근 묶고 있습니다. 조금만 기다려주세요. 먼저 궁금한 점이나 응원의 메시지를 남겨주시면 이후 페이지 구성에 반영하겠습니다.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr" s="2">
+      <c r="O8" t="inlineStr" s="2">
+        <is>
+          <t>The actual workflow, output examples, and verification criteria are being assembled step by step. Please wait a little longer. Questions or messages of support will help shape the next version of the page.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr" s="2">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="2">
+      <c r="Q8" t="inlineStr" s="2">
+        <is>
+          <t>Under construction|Please wait a little longer|A message of support makes a big difference to the next update</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr" s="2">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr" s="2">
+      <c r="S8" t="inlineStr" s="2">
+        <is>
+          <t>Send a message of support</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -814,72 +1357,129 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
+          <t>Image review agent</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
           <t>초상 이미지를 기준으로 클리닝 영역을 감지해서 마킹하고 문서화해주는 에이전트.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="2">
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t>An agent that detects cleanup areas from portrait images, marks them, and documents the review.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
         <is>
           <t>AI agent</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="2">
+      <c r="G9" t="inlineStr" s="2">
+        <is>
+          <t>AI agent</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="2">
         <is>
           <t>공사중</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr" s="2">
+      <c r="I9" t="inlineStr" s="2">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="2">
         <is>
           <t>Review system</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr" s="2">
+      <c r="K9" t="inlineStr" s="2">
+        <is>
+          <t>Review system</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr" s="2">
         <is>
           <t>딸깍클리닝 상세 페이지는 지금 정리 중입니다.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr" s="2">
+      <c r="M9" t="inlineStr" s="2">
+        <is>
+          <t>The TTALKKAK CLEANING detail page is currently being organized.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr" s="2">
         <is>
           <t>클리닝 체크 기준, 마킹 예시, 문서화 흐름을 보기 좋게 정리하는 중입니다. 조금만 기다려주세요. 응원의 메시지나 궁금한 점을 보내주시면 다음 업데이트에 참고하겠습니다.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr" s="2">
+      <c r="O9" t="inlineStr" s="2">
+        <is>
+          <t>The cleanup criteria, marking examples, and documentation flow are being organized for easy review. Please wait a little longer. Messages of support and questions will be considered in the next update.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr" s="2">
         <is>
           <t>공사중|조금만 기다려주세요|응원의 메시지를 보내면 업데이트에 큰 힘이 됩니다</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr" s="2">
+      <c r="Q9" t="inlineStr" s="2">
+        <is>
+          <t>Under construction|Please wait a little longer|A message of support makes a big difference to the next update</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr" s="2">
         <is>
           <t>응원의 메시지 보내기</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr" s="2">
+      <c r="S9" t="inlineStr" s="2">
+        <is>
+          <t>Send a message of support</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M9"/>
+  <autoFilter ref="A1:X9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -890,7 +1490,17 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
+          <t>title_en</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
           <t>summary</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>summary_en</t>
         </is>
       </c>
     </row>
@@ -902,24 +1512,35 @@
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
+          <t>Open Works</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
           <t>다양한 작업들의 아카이빙 및 실험실 공간입니다.</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t>An archive and laboratory for a range of projects.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B2"/>
+  <autoFilter ref="A1:D2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="57" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="57" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -935,10 +1556,15 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>label_en</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>url</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>sort</t>
         </is>
@@ -957,10 +1583,15 @@
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
+          <t>View on GitHub</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
           <t>https://github.com/kyutomatte/sleepless/</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="E2" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -979,10 +1610,15 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
+          <t>Download for macOS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
           <t>/assets/downloads/sleepless/Sleepless_0.1.2_aarch64.dmg</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="E3" t="inlineStr" s="2">
         <is>
           <t>2</t>
         </is>
@@ -1001,10 +1637,15 @@
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
+          <t>Open the web app</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
           <t>/jeju-wave-radio-webapp</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="E4" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1023,10 +1664,15 @@
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
+          <t>Open the web app (beta)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
           <t>/splatify-webapp</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="E5" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1045,10 +1691,15 @@
       </c>
       <c r="C6" t="inlineStr" s="2">
         <is>
+          <t>View on GitHub</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
           <t>https://github.com/kyutomatte/ffMOCHI</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="E6" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1067,10 +1718,15 @@
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
+          <t>Download for macOS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
           <t>/assets/downloads/ffmochi/ffMOCHI-local.dmg</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="E7" t="inlineStr" s="2">
         <is>
           <t>2</t>
         </is>
@@ -1089,32 +1745,40 @@
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
+          <t>View on GitHub</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
           <t>https://github.com/kyutomatte/jebi_agent</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="E8" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:E8"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="56" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="58" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="56" customWidth="1"/>
+    <col min="9" max="9" width="58" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1130,25 +1794,40 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>kicker_en</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>title_en</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>media_url</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>media_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>caption</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>caption_en</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t>sort</t>
         </is>
@@ -1167,25 +1846,40 @@
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
           <t>JEJU WAVE RADIO demo</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="E2" t="inlineStr" s="2">
+        <is>
+          <t>JEJU WAVE RADIO demo</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
         <is>
           <t>/assets/open-works/jeju-wave-radio/jeju-wave-radio-demo.mp4</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
         <is>
           <t>video</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="H2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1204,25 +1898,40 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
           <t>Splatify demo</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>Splatify demo</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
         <is>
           <t>/assets/open-works/splatify/splatify-demo.mov</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="G3" t="inlineStr" s="2">
         <is>
           <t>video</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="H3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1241,46 +1950,64 @@
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
+          <t>Usage example</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
           <t>제비 요청 인식</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>Recognizing a JEBI request</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
         <is>
           <t>/assets/open-works/jebi-agent/jebi-usage-example.png</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="G4" t="inlineStr" s="2">
         <is>
           <t>image</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr" s="2">
+      <c r="H4" t="inlineStr" s="2">
         <is>
           <t>사용자가 제비로 이사갈게요라고 말하면
 JEBI 요청으로 인식하고 handoff 절차를 시작합니다.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="2">
+      <c r="I4" t="inlineStr" s="2">
+        <is>
+          <t>When the user says they want to move with JEBI, the agent recognizes it as a JEBI request and begins the handoff process.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:J4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
+    <col min="6" max="6" width="58" customWidth="1"/>
+    <col min="7" max="7" width="58" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1296,15 +2023,30 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>section_title_en</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>step_title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>step_title_en</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>body</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>body_en</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>sort</t>
         </is>
@@ -1323,15 +2065,30 @@
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
           <t>설치하기</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="E2" t="inlineStr" s="2">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
         <is>
           <t>GitHub Releases 또는 MAC OS용 다운로드 버튼에서 Apple Silicon Mac용 DMG를 받은 뒤 Sleepless.app을 Applications 폴더로 옮겨주세요.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t>Download the DMG for Apple Silicon Macs from GitHub Releases or the Download for macOS button, then move Sleepless.app to the Applications folder.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1350,15 +2107,30 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
           <t>처음 실행 허용하기</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>Allow the first launch</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
         <is>
           <t>개인이 테스트 배포하는 빌드라 아직 Apple 공식 개발자 서명과 공증이 적용되어 있지 않습니다. 안전한 배포 절차를 준비 중이니 처음 실행 시 macOS 보안 안내가 나타날 수 있습니다. 먼저 Done을 눌러 경고창을 닫고, System Settings &gt; Privacy &amp; Security에서 Open Anyway를 선택해주세요. 완료를 누른 뒤 시스템 설정 &gt; 개인정보 보호 및 보안에서 그래도 열기를 선택하면 실행할 수 있습니다. macOS 버전에 따라 버튼 이름이 조금 다를 수 있습니다.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t>This is an individually distributed test build and does not yet have Apple's official developer signature or notarization. A safer distribution process is being prepared, so macOS may show a security notice on first launch. Select Done to close the warning, then choose Open Anyway in System Settings &gt; Privacy &amp; Security. Button names may vary slightly by macOS version.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="2">
         <is>
           <t>2</t>
         </is>
@@ -1377,15 +2149,30 @@
       </c>
       <c r="C4" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
           <t>전원 연결 확인하기</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>Check the power connection</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
         <is>
           <t>SLEEPLESS는 AC 전원 연결 상태에서만 awake mode를 켤 수 있습니다. 전원이 빠지면 배터리 보호를 위해 모드가 자동으로 종료됩니다.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t>SLEEPLESS can enable awake mode only while AC power is connected. If power is disconnected, the mode turns off automatically to protect the battery.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
         <is>
           <t>3</t>
         </is>
@@ -1404,15 +2191,30 @@
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
           <t>잠자기 방지 켜기</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t>Enable sleep prevention</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
         <is>
           <t>메뉴바의 8bit 유령 아이콘에서 잠자기 방지를 켭니다. 처음 켤 때는 closed-lid sleep 제어를 위한 관리자 인증이 한 번 필요할 수 있습니다.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="G5" t="inlineStr" s="2">
+        <is>
+          <t>Use the 8-bit ghost icon in the menu bar to enable sleep prevention. The first time you turn it on, macOS may require administrator authentication to control closed-lid sleep.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="2">
         <is>
           <t>4</t>
         </is>
@@ -1431,15 +2233,30 @@
       </c>
       <c r="C6" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
           <t>유지 시간 고르기</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t>Choose the duration</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
         <is>
           <t>닫힌 상태 유지 시간을 10분, 30분, 1시간, 영구 중에서 고를 수 있습니다. 뚜껑을 닫으면 밝기를 0으로 낮추고, 다시 열거나 모드를 끄면 이전 밝기를 복구합니다.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="G6" t="inlineStr" s="2">
+        <is>
+          <t>Choose 10 minutes, 30 minutes, 1 hour, or indefinitely for the closed-lid duration. When the lid closes, brightness drops to zero; opening the lid or turning off the mode restores the previous brightness.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="2">
         <is>
           <t>5</t>
         </is>
@@ -1458,15 +2275,30 @@
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
+          <t>SLEEPLESS Manual</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
           <t>문제 시 복구하기</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t>Recover from problems</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
         <is>
           <t>앱이 비정상 종료된 뒤 닫힘 잠자기가 돌아오지 않으면 터미널에서 sudo pmset -c disablesleep 0 명령으로 macOS 기본 전원 설정을 복구할 수 있습니다.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="2">
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t>If normal closed-lid sleep does not return after the app exits unexpectedly, run sudo pmset -c disablesleep 0 in Terminal to restore the default macOS power setting.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="2">
         <is>
           <t>6</t>
         </is>
@@ -1485,15 +2317,30 @@
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
           <t>설치하기</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
         <is>
           <t>MAC OS용 다운로드 버튼에서 ffMOCHI-local.dmg를 받은 뒤 ffMOCHI.app을 Applications 폴더로 드래그해주세요.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="2">
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t>Download ffMOCHI-local.dmg using the Download for macOS button, then drag ffMOCHI.app to the Applications folder.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1512,15 +2359,30 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
           <t>처음 실행 허용하기</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="2">
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t>Allow the first launch</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
         <is>
           <t>개인이 테스트 배포하는 빌드라 아직 Apple 공식 개발자 서명과 공증이 적용되어 있지 않습니다. 안전한 배포 절차를 준비 중이니 처음 실행 시 macOS 보안 안내가 나타날 수 있습니다. 먼저 Done을 눌러 경고창을 닫고, System Settings &gt; Privacy &amp; Security에서 Open Anyway를 선택해주세요. 완료를 누른 뒤 시스템 설정 &gt; 개인정보 보호 및 보안에서 그래도 열기를 선택하면 실행할 수 있습니다. macOS 버전에 따라 버튼 이름이 조금 다를 수 있습니다.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="2">
+      <c r="G9" t="inlineStr" s="2">
+        <is>
+          <t>This is an individually distributed test build and does not yet have Apple's official developer signature or notarization. A safer distribution process is being prepared, so macOS may show a security notice on first launch. Select Done to close the warning, then choose Open Anyway in System Settings &gt; Privacy &amp; Security. Button names may vary slightly by macOS version.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="2">
         <is>
           <t>2</t>
         </is>
@@ -1539,15 +2401,30 @@
       </c>
       <c r="C10" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
           <t>FFmpeg 준비하기</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="2">
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t>Prepare FFmpeg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
         <is>
           <t>ffMOCHI는 로컬 FFmpeg로 영상을 압축합니다. 앱에 설치 안내가 보이면 Homebrew에서 brew install ffmpeg를 실행한 뒤 CHECK AGAIN을 눌러주세요.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="2">
+      <c r="G10" t="inlineStr" s="2">
+        <is>
+          <t>ffMOCHI compresses video with a local FFmpeg installation. If the app shows an installation notice, run brew install ffmpeg with Homebrew, then select CHECK AGAIN.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="2">
         <is>
           <t>3</t>
         </is>
@@ -1566,15 +2443,30 @@
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
           <t>영상 넣고 시작하기</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr" s="2">
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t>Add a video and start</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
         <is>
           <t>MP4 MOV M4V 파일을 앱 창에 드래그하거나 앱 아이콘 위에 드롭한 뒤 프리셋을 고르고 START를 누르면 압축이 시작됩니다.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="2">
+      <c r="G11" t="inlineStr" s="2">
+        <is>
+          <t>Drag an MP4, MOV, or M4V file into the app window or drop it onto the app icon, choose a preset, and select START to begin compression.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr" s="2">
         <is>
           <t>4</t>
         </is>
@@ -1593,15 +2485,30 @@
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
           <t>출력 확인하기</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="2">
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t>Check the output</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="2">
         <is>
           <t>완료된 파일은 원본 옆에 OriginalName_compressed.mp4 형태로 저장됩니다. 같은 이름이 있으면 _compressed_001.mp4처럼 번호를 붙여 덮어쓰지 않습니다.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="2">
+      <c r="G12" t="inlineStr" s="2">
+        <is>
+          <t>The completed file is saved beside the original as OriginalName_compressed.mp4. If that name already exists, a number such as _compressed_001.mp4 is added so nothing is overwritten.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr" s="2">
         <is>
           <t>5</t>
         </is>
@@ -1620,15 +2527,30 @@
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
+          <t>ffMOCHI Manual</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
           <t>문제 시 확인하기</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="2">
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t>Troubleshooting</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="2">
         <is>
           <t>압축이 실패하면 FFmpeg 설치, 지원 파일 형식, 출력 폴더 권한, 디스크 공간을 확인해주세요. Default MP4로 다시 시도하기 전 일부만 만들어진 _compressed.mp4 파일이 남아 있으면 삭제하는 것이 좋습니다.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="2">
+      <c r="G13" t="inlineStr" s="2">
+        <is>
+          <t>If compression fails, check the FFmpeg installation, supported file format, output-folder permissions, and available disk space. Before retrying with Default MP4, it is best to remove any partial _compressed.mp4 file.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr" s="2">
         <is>
           <t>6</t>
         </is>
@@ -1647,15 +2569,30 @@
       </c>
       <c r="C14" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
           <t>왜 필요한가</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="2">
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t>Why you need it</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="2">
         <is>
           <t>긴 코딩 채팅이 무거워지고 컨텍스트가 길어져 결정이 묻히기 시작할 때 씁니다. Fork는 너무 많은 history를 복사하고, 완전히 새로 시작하면 맥락을 잃습니다. JEBI는 그 중간 지점에서 현재 작업 상태만 압축해 새 채팅으로 넘깁니다.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="2">
+      <c r="G14" t="inlineStr" s="2">
+        <is>
+          <t>Use JEBI when a long coding chat becomes heavy and important decisions start getting buried in the growing context. A fork copies too much history, while starting from scratch loses the context. JEBI takes the middle path by compressing only the current work state and passing it to a new chat.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr" s="2">
         <is>
           <t>1</t>
         </is>
@@ -1674,16 +2611,32 @@
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
           <t>설치와 발동</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="2">
+      <c r="E15" t="inlineStr" s="2">
+        <is>
+          <t>Install and trigger</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="2">
         <is>
           <t>가장 쉬운 설치 방법은 GitHub 주소와 README를 에이전트에게 전달하는 것입니다. 단, 주소만 주는 방식은 해당 대화 안에서 읽고 따라 하는 것에 가깝습니다. 다음 대화에서도 자동으로 JEBI가 발동되게 하려면 사용하는 도구가 지원하는 Skills, 프로젝트 지침, custom instruction 중 하나에 등록해야 합니다.
 PROMPT: https://github.com/kyutomatte/jebi_agent 확인하고 README.md 기준으로 설치와 사용 방법을 알려주세요.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr" s="2">
+      <c r="G15" t="inlineStr" s="2">
+        <is>
+          <t>The easiest installation method is to give the agent the GitHub URL and README. Providing only the URL, however, is closer to asking the agent to read and follow it in that conversation. To trigger JEBI automatically in future conversations, register it in one of the supported mechanisms: Skills, project instructions, or custom instructions.
+PROMPT: Review https://github.com/kyutomatte/jebi_agent and explain how to install and use it according to README.md.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr" s="2">
         <is>
           <t>2</t>
         </is>
@@ -1702,10 +2655,20 @@
       </c>
       <c r="C16" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
           <t>환경별 설치 방법</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr" s="2">
+      <c r="E16" t="inlineStr" s="2">
+        <is>
+          <t>Installation by environment</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="2">
         <is>
           <t>환경|가장 쉬운 방법|계속 쓰는 방법|발동 문구
 ChatGPT / GPT|GitHub 주소와 README.md를 읽어 달라고 합니다.|지원되는 Skills/프로젝트 지침 환경이면 Skill 폴더 또는 SKILL.md 핵심 규칙을 등록하고, 일반 ChatGPT/GPT에서는 Custom Instructions, GPT 지침, 프로젝트 지침에 핵심 규칙을 붙입니다.|$jebi 또는 제비로 옮겨주세요
@@ -1716,7 +2679,18 @@
 기타 LLM|GitHub 주소를 주고 README.md를 따라 하게 합니다.|system/custom instruction, 프로젝트 지침, 지식 베이스에 SKILL.md 핵심을 넣습니다.|JEBI 모드로 정리해줘</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr" s="2">
+      <c r="G16" t="inlineStr" s="2">
+        <is>
+          <t>Environment|Easiest method|Persistent setup|Trigger phrase
+ChatGPT / GPT|Ask it to read the GitHub URL and README.md.|In environments that support Skills or project instructions, register the Skill folder or the core SKILL.md rules. In standard ChatGPT/GPT, add the core rules to Custom Instructions, GPT instructions, or project instructions.|$jebi or move this with JEBI
+Codex|Clone this repo and follow the Codex installation steps in the README.|Place the Skill folders at ~/.codex/skills/jebi-agent and ~/.codex/skills/jebi. To make it available automatically for a project, you can also add the JEBI invocation rule to AGENTS.md.|$jebi or move this with JEBI
+Claude app|Provide the GitHub URL and ask it to follow the instructions in the current conversation.|Upload the Skill folder only in environments with a Skill upload UI. Otherwise add the core SKILL.md rules to Project knowledge or custom instructions.|use the jebi-agent skill or move this with a JEBI handoff
+Claude Code|Clone this repo and run the terminal installation command.|Place the Skill folder at ~/.claude/skills/jebi-agent or the project's .claude/skills/jebi-agent.|/jebi-agent
+Gemini CLI|Ask it to read the GitHub URL or the contents of SKILL.md.|Run scripts/install-skill.sh gemini to install the .toml-based custom command. Run /commands reload if needed.|/jebi or /jebi move the current work to a new chat
+Other LLM|Provide the GitHub URL and ask it to follow README.md.|Add the core SKILL.md rules to system/custom instructions, project instructions, or a knowledge base.|Summarize this in JEBI mode</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr" s="2">
         <is>
           <t>3</t>
         </is>
@@ -1735,10 +2709,20 @@
       </c>
       <c r="C17" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
           <t>터미널 설치</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="2">
+      <c r="E17" t="inlineStr" s="2">
+        <is>
+          <t>Terminal installation</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr" s="2">
         <is>
           <t>터미널에서 쓰는 에이전트는 설치 스크립트가 가장 단순합니다.
 CMD: scripts/install-skill.sh codex
@@ -1753,7 +2737,22 @@
 지침, custom command, 프로젝트 rule은 설치할 수 있지만 Codex Desktop thread API가 생기지는 않습니다.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr" s="2">
+      <c r="G17" t="inlineStr" s="2">
+        <is>
+          <t>For terminal-based agents, the installation script is the simplest option.
+CMD: scripts/install-skill.sh codex
+scripts/install-skill.sh claude
+scripts/install-skill.sh gemini
+scripts/install-skill.sh cursor
+To install everything:
+CMD: scripts/install-skill.sh all
+If Gemini CLI cannot read Skill folders directly, use a custom command.
+CMD: scripts/install-skill.sh gemini
+Gemini and Cursor are best-effort adapters.
+They can install instructions, custom commands, and project rules, but they do not gain access to the Codex Desktop thread API.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr" s="2">
         <is>
           <t>4</t>
         </is>
@@ -1772,10 +2771,20 @@
       </c>
       <c r="C18" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="2">
+        <is>
           <t>호출 예시</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr" s="2">
+      <c r="E18" t="inlineStr" s="2">
+        <is>
+          <t>Invocation examples</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="2">
         <is>
           <t>유형|예시|설명
 실행어 호출 예시|$jebi|현재 작업을 새 Codex 채팅으로 넘기는 JEBI handoff를 시작합니다.
@@ -1787,7 +2796,19 @@
 오작동 방지|파일명 jebi 또는 동물 제비 이야기|새 채팅 이동 의도가 없으면 실행하지 않습니다.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr" s="2">
+      <c r="G18" t="inlineStr" s="2">
+        <is>
+          <t>Type|Example|Description
+Explicit trigger example|$jebi|Starts a JEBI handoff that transfers the current work to a new Codex chat.
+Explicit trigger example|$jebi-agent|Explicitly invokes JEBI AGENT in the same way.
+Natural-language example|Move this with JEBI|Recognized as a request to continue the current work in a clean new chat.
+Natural-language example|Hand this off with JEBI|Creates a handoff file and prepares the next agent to take over.
+Natural-language example|JEBI, depart|Starts the JEBI process with a short imperative request.
+Natural-language example|Send JEBI to a new chat|Runs when the intention to create a new successor chat is clear.
+False-positive prevention|A file named jebi or a discussion of the swallow bird|Does not run when there is no intent to move to a new chat.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr" s="2">
         <is>
           <t>5</t>
         </is>
@@ -1806,17 +2827,34 @@
       </c>
       <c r="C19" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="2">
+        <is>
           <t>자동으로 넘기는 정보</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="2">
+      <c r="E19" t="inlineStr" s="2">
+        <is>
+          <t>Information transferred automatically</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr" s="2">
         <is>
           <t>JEBI는 현재 repository, branch, HEAD, worktree 상태를 먼저 확인합니다.
 handoff에는 전체 diff가 아니라 변경 파일 요약, 완료한 일과 남은 일, 중요한 결정, 바꾸면 안 되는 내용이 들어갑니다.
 test/build/lint/typecheck 상태, 적용되는 AGENTS.md 지침, known failure recovery note도 함께 정리합니다.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr" s="2">
+      <c r="G19" t="inlineStr" s="2">
+        <is>
+          <t>JEBI first checks the current repository, branch, HEAD, and worktree state.
+The handoff contains a summary of changed files, completed and remaining work, important decisions, and things that must not change rather than the full diff.
+It also records test/build/lint/typecheck status, applicable AGENTS.md instructions, and known failure-recovery notes.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr" s="2">
         <is>
           <t>6</t>
         </is>
@@ -1835,10 +2873,20 @@
       </c>
       <c r="C20" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr" s="2">
+        <is>
           <t>작동 방식</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr" s="2">
+      <c r="E20" t="inlineStr" s="2">
+        <is>
+          <t>How it works</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr" s="2">
         <is>
           <t>실행되면 .codex/handoffs/NNN-handoff.md를 만들고 latest.md를 갱신합니다.
 state.json은 retry와 numbering을 위한 로컬 상태로 남깁니다.
@@ -1846,7 +2894,15 @@
 새 채팅에는 handoff 경로와 확인 지시만 보냅니다.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr" s="2">
+      <c r="G20" t="inlineStr" s="2">
+        <is>
+          <t>When invoked, JEBI creates .codex/handoffs/NNN-handoff.md and updates latest.md.
+state.json remains as local state for retries and numbering.
+In Codex Desktop, it starts a clean successor chat through thread/start or an official thread tool rather than forking.
+The new chat receives only the handoff path and verification instructions.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr" s="2">
         <is>
           <t>7</t>
         </is>
@@ -1865,17 +2921,34 @@
       </c>
       <c r="C21" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr" s="2">
+        <is>
           <t>새 채팅 이름</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr" s="2">
+      <c r="E21" t="inlineStr" s="2">
+        <is>
+          <t>Naming the new chat</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr" s="2">
         <is>
           <t>새 채팅 이름은 프로젝트 폴더명이 아니라 현재 작업 제목을 기준으로 붙입니다. 예를 들어 UI UX에서 처음 옮기면 UI UX #02가 됩니다.
 거기서 다시 옮기면 UI UX #02 #02가 아니라 UI UX #03이 됩니다.
 제목을 읽을 수 없으면 project name으로 대체하지 않습니다.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr" s="2">
+      <c r="G21" t="inlineStr" s="2">
+        <is>
+          <t>The new chat is named after the current task title, not the project folder. For example, the first move from UI UX becomes UI UX #02.
+Moving again from there produces UI UX #03, not UI UX #02 #02.
+If the title cannot be read, JEBI does not substitute the project name.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr" s="2">
         <is>
           <t>8</t>
         </is>
@@ -1894,17 +2967,34 @@
       </c>
       <c r="C22" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr" s="2">
+        <is>
           <t>새 채팅에서 먼저 하는 일</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr" s="2">
+      <c r="E22" t="inlineStr" s="2">
+        <is>
+          <t>What happens first in the new chat</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr" s="2">
         <is>
           <t>successor 에이전트는 handoff 파일을 읽고 실제 repo와 비교합니다.
 브랜치, 워킹트리, 변경 파일, 누락된 맥락이 맞는지 확인하고, 불일치가 있으면 먼저 보고합니다.
 그 전에는 파일을 수정하지 않고 사용자 지시를 기다립니다.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr" s="2">
+      <c r="G22" t="inlineStr" s="2">
+        <is>
+          <t>The successor agent reads the handoff file and compares it with the live repo.
+It checks that the branch, worktree, changed files, and missing context match, and reports any discrepancy first.
+Until then, it does not modify files and waits for user direction.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr" s="2">
         <is>
           <t>9</t>
         </is>
@@ -1923,17 +3013,34 @@
       </c>
       <c r="C23" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr" s="2">
+        <is>
           <t>Dirty 상태 다루기</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr" s="2">
+      <c r="E23" t="inlineStr" s="2">
+        <is>
+          <t>Handling a dirty worktree</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr" s="2">
         <is>
           <t>JEBI는 .codex/handoffs 안에 markdown handoff를 만들기 때문에 실행 직후 dirty 상태가 생길 수 있습니다.
 handoff만 바뀌었다면 Clean except JEBI handoff artifacts로 보고합니다.
 실제 프로젝트 변경과 섞여 있다면 Dirty: project changes + JEBI handoff artifacts로 구분합니다.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr" s="2">
+      <c r="G23" t="inlineStr" s="2">
+        <is>
+          <t>Because JEBI creates a Markdown handoff in .codex/handoffs, the worktree may become dirty immediately after it runs.
+If only the handoff changed, it reports Clean except JEBI handoff artifacts.
+If those artifacts are mixed with project changes, it reports Dirty: project changes + JEBI handoff artifacts.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr" s="2">
         <is>
           <t>10</t>
         </is>
@@ -1952,17 +3059,34 @@
       </c>
       <c r="C24" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr" s="2">
+        <is>
           <t>주의점</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr" s="2">
+      <c r="E24" t="inlineStr" s="2">
+        <is>
+          <t>Important notes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr" s="2">
         <is>
           <t>JEBI는 fork가 아닙니다. 현재 채팅을 복제하는 대신 clean successor chat을 시작합니다.
 전체 이전 채팅 history를 복사하지 않고, AppleScript, 화면 좌표 클릭, 내부 DB 수정, undocumented UI API 같은 우회도 쓰지 않아야 합니다.
 실제 저장소 상태가 대화 기억보다 우선입니다.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr" s="2">
+      <c r="G24" t="inlineStr" s="2">
+        <is>
+          <t>JEBI is not a fork. It starts a clean successor chat instead of copying the current chat.
+It does not copy the full previous chat history and must not use workarounds such as AppleScript, screen-coordinate clicks, internal database edits, or undocumented UI APIs.
+The live repository state takes precedence over conversational memory.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr" s="2">
         <is>
           <t>11</t>
         </is>
@@ -1981,17 +3105,34 @@
       </c>
       <c r="C25" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr" s="2">
+        <is>
           <t>보안 규칙</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr" s="2">
+      <c r="E25" t="inlineStr" s="2">
+        <is>
+          <t>Security rules</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr" s="2">
         <is>
           <t>handoff에는 API keys, tokens, cookies, authorization headers, .env values 같은 민감한 정보를 넣지 않습니다.
 의심되는 값은 REDACTED로 치환합니다.
 파괴적인 git 명령은 사용자 승인 없이 실행하지 않고, 새 채팅이 보이지 않으면 성공으로 말하지 않습니다.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr" s="2">
+      <c r="G25" t="inlineStr" s="2">
+        <is>
+          <t>The handoff does not include sensitive information such as API keys, tokens, cookies, authorization headers, or .env values.
+Suspected values are replaced with REDACTED.
+Destructive git commands are not run without user approval, and JEBI does not claim success unless the new chat is visible.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr" s="2">
         <is>
           <t>12</t>
         </is>
@@ -2010,23 +3151,40 @@
       </c>
       <c r="C26" t="inlineStr" s="2">
         <is>
+          <t>JEBI AGENT Tutorial</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr" s="2">
+        <is>
           <t>테스트와 삭제</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr" s="2">
+      <c r="E26" t="inlineStr" s="2">
+        <is>
+          <t>Testing and removal</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr" s="2">
         <is>
           <t>개발자는 python3 -m unittest discover -s tests -v로 루트 테스트를 돌립니다.
 Skill 번들 테스트는 python3 -m unittest discover -s skill/jebi-agent/tests -v로 확인합니다.
 삭제할 때는 rm -rf ~/.codex/skills/jebi-agent 와 rm -rf ~/.codex/skills/jebi를 실행합니다. 프로젝트의 handoff 파일은 별도로 남습니다.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr" s="2">
+      <c r="G26" t="inlineStr" s="2">
+        <is>
+          <t>Developers run the root tests with python3 -m unittest discover -s tests -v.
+Run the Skill bundle tests with python3 -m unittest discover -s skill/jebi-agent/tests -v.
+To remove the Skills, run rm -rf ~/.codex/skills/jebi-agent and rm -rf ~/.codex/skills/jebi. Project handoff files remain separately.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr" s="2">
         <is>
           <t>13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:H26"/>
 </worksheet>
 </file>
</xml_diff>